<commit_message>
update states and communes
</commit_message>
<xml_diff>
--- a/lib/assets/states___14_07_2025.xlsx
+++ b/lib/assets/states___14_07_2025.xlsx
@@ -45,114 +45,63 @@
     <t>04</t>
   </si>
   <si>
-    <t>Cao Bằng</t>
-  </si>
-  <si>
     <t>Tỉnh</t>
   </si>
   <si>
     <t>08</t>
   </si>
   <si>
-    <t>Tuyên Quang</t>
-  </si>
-  <si>
     <t xml:space="preserve">202/2025/QH15 - 12/06/2025                    </t>
   </si>
   <si>
     <t>11</t>
   </si>
   <si>
-    <t>Điện Biên</t>
-  </si>
-  <si>
     <t>12</t>
   </si>
   <si>
-    <t>Lai Châu</t>
-  </si>
-  <si>
     <t>14</t>
   </si>
   <si>
-    <t>Sơn La</t>
-  </si>
-  <si>
     <t>15</t>
   </si>
   <si>
-    <t>Lào Cai</t>
-  </si>
-  <si>
     <t>19</t>
   </si>
   <si>
-    <t>Thái Nguyên</t>
-  </si>
-  <si>
     <t>20</t>
   </si>
   <si>
-    <t>Lạng Sơn</t>
-  </si>
-  <si>
     <t>22</t>
   </si>
   <si>
-    <t>Quảng Ninh</t>
-  </si>
-  <si>
     <t>24</t>
   </si>
   <si>
-    <t>Bắc Ninh</t>
-  </si>
-  <si>
     <t>25</t>
   </si>
   <si>
-    <t>Phú Thọ</t>
-  </si>
-  <si>
     <t>31</t>
   </si>
   <si>
     <t>33</t>
   </si>
   <si>
-    <t>Hưng Yên</t>
-  </si>
-  <si>
     <t>37</t>
   </si>
   <si>
-    <t>Ninh Bình</t>
-  </si>
-  <si>
     <t>38</t>
   </si>
   <si>
-    <t>Thanh Hóa</t>
-  </si>
-  <si>
     <t>40</t>
   </si>
   <si>
-    <t>Nghệ An</t>
-  </si>
-  <si>
     <t>42</t>
   </si>
   <si>
-    <t>Hà Tĩnh</t>
-  </si>
-  <si>
     <t>44</t>
   </si>
   <si>
-    <t>Quảng Trị</t>
-  </si>
-  <si>
     <t>46</t>
   </si>
   <si>
@@ -162,91 +111,142 @@
     <t>51</t>
   </si>
   <si>
-    <t>Quảng Ngãi</t>
-  </si>
-  <si>
     <t>52</t>
   </si>
   <si>
-    <t>Gia Lai</t>
-  </si>
-  <si>
     <t>56</t>
   </si>
   <si>
-    <t>Khánh Hòa</t>
-  </si>
-  <si>
     <t>66</t>
   </si>
   <si>
-    <t>Đắk Lắk</t>
-  </si>
-  <si>
     <t>68</t>
   </si>
   <si>
-    <t>Lâm Đồng</t>
-  </si>
-  <si>
     <t>75</t>
   </si>
   <si>
-    <t>Đồng Nai</t>
-  </si>
-  <si>
     <t>79</t>
   </si>
   <si>
     <t>80</t>
   </si>
   <si>
-    <t>Tây Ninh</t>
-  </si>
-  <si>
     <t>82</t>
   </si>
   <si>
-    <t>Đồng Tháp</t>
-  </si>
-  <si>
     <t>86</t>
   </si>
   <si>
-    <t>Vĩnh Long</t>
-  </si>
-  <si>
     <t>91</t>
   </si>
   <si>
-    <t>An Giang</t>
-  </si>
-  <si>
     <t>92</t>
   </si>
   <si>
     <t>96</t>
   </si>
   <si>
-    <t>Cà Mau</t>
-  </si>
-  <si>
-    <t>Hà Nội</t>
-  </si>
-  <si>
-    <t>Hải Phòng</t>
-  </si>
-  <si>
-    <t>Huế</t>
-  </si>
-  <si>
-    <t>Đà Nẵng</t>
-  </si>
-  <si>
     <t>Thành phố Hồ Chí Minh</t>
   </si>
   <si>
-    <t>Cần Thơ</t>
+    <t>Thành phố Hà Nội</t>
+  </si>
+  <si>
+    <t>Thành phố Hải Phòng</t>
+  </si>
+  <si>
+    <t>Thành phố Huế</t>
+  </si>
+  <si>
+    <t>Thành phố Đà Nẵng</t>
+  </si>
+  <si>
+    <t>Thành phố Cần Thơ</t>
+  </si>
+  <si>
+    <t>Tỉnh Cao Bằng</t>
+  </si>
+  <si>
+    <t>Tỉnh Tuyên Quang</t>
+  </si>
+  <si>
+    <t>Tỉnh Điện Biên</t>
+  </si>
+  <si>
+    <t>Tỉnh Lai Châu</t>
+  </si>
+  <si>
+    <t>Tỉnh Sơn La</t>
+  </si>
+  <si>
+    <t>Tỉnh Lào Cai</t>
+  </si>
+  <si>
+    <t>Tỉnh Thái Nguyên</t>
+  </si>
+  <si>
+    <t>Tỉnh Lạng Sơn</t>
+  </si>
+  <si>
+    <t>Tỉnh Quảng Ninh</t>
+  </si>
+  <si>
+    <t>Tỉnh Bắc Ninh</t>
+  </si>
+  <si>
+    <t>Tỉnh Phú Thọ</t>
+  </si>
+  <si>
+    <t>Tỉnh Hưng Yên</t>
+  </si>
+  <si>
+    <t>Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>Tỉnh Thanh Hóa</t>
+  </si>
+  <si>
+    <t>Tỉnh Nghệ An</t>
+  </si>
+  <si>
+    <t>Tỉnh Hà Tĩnh</t>
+  </si>
+  <si>
+    <t>Tỉnh Quảng Trị</t>
+  </si>
+  <si>
+    <t>Tỉnh Quảng Ngãi</t>
+  </si>
+  <si>
+    <t>Tỉnh Gia Lai</t>
+  </si>
+  <si>
+    <t>Tỉnh Khánh Hòa</t>
+  </si>
+  <si>
+    <t>Tỉnh Đắk Lắk</t>
+  </si>
+  <si>
+    <t>Tỉnh Lâm Đồng</t>
+  </si>
+  <si>
+    <t>Tỉnh Đồng Nai</t>
+  </si>
+  <si>
+    <t>Tỉnh Tây Ninh</t>
+  </si>
+  <si>
+    <t>Tỉnh Đồng Tháp</t>
+  </si>
+  <si>
+    <t>Tỉnh Vĩnh Long</t>
+  </si>
+  <si>
+    <t>Tỉnh An Giang</t>
+  </si>
+  <si>
+    <t>Tỉnh Cà Mau</t>
   </si>
 </sst>
 </file>
@@ -948,7 +948,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
@@ -961,478 +961,478 @@
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E20" s="2"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="2"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" s="2"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E31" s="2"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E33" s="2"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>